<commit_message>
FEAT: add custom Capacity
</commit_message>
<xml_diff>
--- a/input/MaterialData.xlsx
+++ b/input/MaterialData.xlsx
@@ -4,18 +4,19 @@
   <fileVersion appName="Polaris Office Sheet" lastEdited="4" lowestEdited="4" rupBuild=""/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="4"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="FlowName" sheetId="1" r:id="rId1"/>
     <sheet name="Except Unit" sheetId="2" r:id="rId2"/>
-    <sheet name="Reactor" sheetId="3" r:id="rId3"/>
-    <sheet name="Equipment Cost Parameter" sheetId="4" r:id="rId4"/>
-    <sheet name="Utility Parameter" sheetId="5" r:id="rId5"/>
-    <sheet name="input" sheetId="6" r:id="rId6"/>
-    <sheet name="output" sheetId="7" r:id="rId7"/>
-    <sheet name="Example input data" sheetId="8" r:id="rId8"/>
-    <sheet name="Example output data" sheetId="9" r:id="rId9"/>
+    <sheet name="Capacity" sheetId="10" r:id="rId3"/>
+    <sheet name="Reactor" sheetId="3" r:id="rId4"/>
+    <sheet name="Equipment Cost Parameter" sheetId="4" r:id="rId5"/>
+    <sheet name="Utility Parameter" sheetId="5" r:id="rId6"/>
+    <sheet name="input" sheetId="6" r:id="rId7"/>
+    <sheet name="output" sheetId="7" r:id="rId8"/>
+    <sheet name="Example input data" sheetId="8" r:id="rId9"/>
+    <sheet name="Example output data" sheetId="9" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="152511"/>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
   <si>
     <t>Reactor Name</t>
   </si>
@@ -263,6 +264,18 @@
   </si>
   <si>
     <t>StreamPrice(MPS)</t>
+  </si>
+  <si>
+    <t>EquipmentName</t>
+  </si>
+  <si>
+    <t>Capacity[KW, M^2]</t>
+  </si>
+  <si>
+    <t>Capacity [KW, M^2]</t>
+  </si>
+  <si>
+    <t>Equipment Name</t>
   </si>
 </sst>
 </file>
@@ -2496,6 +2509,233 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:D20"/>
+  <sheetFormatPr defaultRowHeight="13.200000"/>
+  <cols>
+    <col min="2" max="2" width="15.38000011" customWidth="1" outlineLevel="0"/>
+    <col min="3" max="3" width="24.12999916" customWidth="1" outlineLevel="0"/>
+    <col min="4" max="4" width="23.00499916" customWidth="1" outlineLevel="0"/>
+    <col min="5" max="5" width="12.13000011" customWidth="1" outlineLevel="0"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="B3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4">
+      <c r="B4" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="B5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="B6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="B7" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="B8" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="B9" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4">
+      <c r="B10" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4">
+      <c r="B11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="B12" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="B13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="B14" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="B15" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="B16" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4">
+      <c r="B19" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="B20" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C20" s="10">
+        <v>0.325</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:D3"/>
@@ -2527,6 +2767,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="B2:C2"/>
+  <sheetFormatPr defaultRowHeight="13.200000"/>
+  <cols>
+    <col min="2" max="2" width="18.50499916" customWidth="1" outlineLevel="0"/>
+    <col min="3" max="3" width="25.75499916" customWidth="1" outlineLevel="0"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3">
+      <c r="B2" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:C7"/>
   <sheetFormatPr defaultRowHeight="13.200000"/>
   <cols>
@@ -2589,7 +2853,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:H18"/>
   <sheetFormatPr defaultRowHeight="13.200000"/>
@@ -2795,7 +3059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:AH14"/>
   <sheetFormatPr defaultRowHeight="13.200000"/>
@@ -2923,7 +3187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AJ40"/>
   <sheetFormatPr defaultColWidth="8.83333000" defaultRowHeight="15.000000" customHeight="1"/>
@@ -4418,7 +4682,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:P20"/>
   <sheetFormatPr defaultRowHeight="13.200000"/>
@@ -4766,7 +5030,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="B2:D6"/>
   <sheetFormatPr defaultRowHeight="13.200000"/>
@@ -4826,231 +5090,4 @@
   <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B2:D20"/>
-  <sheetFormatPr defaultRowHeight="13.200000"/>
-  <cols>
-    <col min="2" max="2" width="15.38000011" customWidth="1" outlineLevel="0"/>
-    <col min="3" max="3" width="24.12999916" customWidth="1" outlineLevel="0"/>
-    <col min="4" max="4" width="23.00499916" customWidth="1" outlineLevel="0"/>
-    <col min="5" max="5" width="12.13000011" customWidth="1" outlineLevel="0"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:4">
-      <c r="B2" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4">
-      <c r="B3" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4">
-      <c r="B4" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C4" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4">
-      <c r="B5" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4">
-      <c r="B6" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4">
-      <c r="B7" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4">
-      <c r="B8" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4">
-      <c r="B9" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4">
-      <c r="B10" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4">
-      <c r="B11" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4">
-      <c r="B12" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4">
-      <c r="B13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4">
-      <c r="B14" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4">
-      <c r="B15" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4">
-      <c r="B16" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C16" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4">
-      <c r="B17" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4">
-      <c r="B18" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D18" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="2:4">
-      <c r="B19" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C19" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D19" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="2:4">
-      <c r="B20" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C20" s="10">
-        <v>0.325</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>60</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.70" right="0.70" top="0.75" bottom="0.75" header="0.30" footer="0.30"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
 </file>
</xml_diff>